<commit_message>
Fix KURIS/NDD scores to match figure data
</commit_message>
<xml_diff>
--- a/data/output/BAP1_Missense_Variants_Combined.xlsx
+++ b/data/output/BAP1_Missense_Variants_Combined.xlsx
@@ -536,16 +536,16 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>p.Cys91Ser</t>
+          <t>p.Asn229Lys</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>c.272G&gt;C</t>
+          <t>c.687C&gt;A</t>
         </is>
       </c>
       <c r="D3" t="n">
-        <v>-0.176975473</v>
+        <v>-0.2001695</v>
       </c>
       <c r="E3" t="inlineStr">
         <is>
@@ -554,33 +554,33 @@
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>Pathogenic</t>
+          <t>Likely pathogenic</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>VCV001173081</t>
+          <t>VCV002429331</t>
         </is>
       </c>
       <c r="H3" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>SCV001738372: P, Cond: Neurodevelopmental disorder, MedGenet, 2021-06-22 [de novo; affected: yes]</t>
-        </is>
-      </c>
-      <c r="J3" t="inlineStr">
-        <is>
-          <t>F5 (Sex: female; Age_at_last_investigation: 11 years 5 months; Growth_failure: +; Developmental_delay_or_ID: +; severe; Seizures: +; Urogenital_kidney_anomalies: +; Feet: +; Facial_dysmorphism: +; Other_recurrent_signs: hypertrichosis)</t>
-        </is>
-      </c>
+          <t>SCV003799185: LP, IHG-UKRWTH, 2023-02-09 [de novo; affected: yes; To our knowledge, the variant has not yet been described in the literature. Küry S. et al. (2022) describe 11 individuals with a similar phenotype to our patient with de novo missense variants in BAP1, which are also located d in a protein domain that encodes for a ubiquitin carboxyl-terminal hydrolase (peptidase C12) and the papain-like cysteine ​​peptidase superfamily. Functional studies of these variants show that they alter chromatin remodeling through abnormal histone ubiquitination and result in transcriptional dysregulation of developmental genes. (PMID: 35051358) These findings suggest that this could also lead to defective histone ubiquitination in the variant described here.]; SCV006550944: LP, UDN, 2025-06-11 [de novo; affected: yes; clinical features: Hearing impairment, Short neck, Cataract, Retinal detachment, Leukocoria, Microphthalmia, Shallow anterior chamber, Brachydactyly, Global developmental delay, Sandal gap, Bilateral retinal detachment, Hallux valgus]</t>
+        </is>
+      </c>
+      <c r="J3" t="inlineStr"/>
       <c r="K3" t="inlineStr">
         <is>
-          <t>44493 (GDX)</t>
-        </is>
-      </c>
-      <c r="L3" t="inlineStr"/>
+          <t>DDD13k.05634 (DDD)</t>
+        </is>
+      </c>
+      <c r="L3" t="inlineStr">
+        <is>
+          <t>Patient 264575 (46XY; De novo (parentage confirmed)) [3-4 finger osseus syndactyly; Abnormal forehead morphology; Abnormal nail morphology; Broad forehead; Cutaneous finger syndactyly; Delayed gross motor development; Delayed speech and language development; Global developmental delay; Hypermetropia; Microdontia; Short stature; Upslanted palpebral fissure]</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -590,16 +590,16 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>p.His169Gln</t>
+          <t>p.Cys91Ser</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>c.507C&gt;G</t>
+          <t>c.272G&gt;C</t>
         </is>
       </c>
       <c r="D4" t="n">
-        <v>-0.1688213</v>
+        <v>-0.176975473</v>
       </c>
       <c r="E4" t="inlineStr">
         <is>
@@ -608,12 +608,12 @@
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>Likely pathogenic</t>
+          <t>Pathogenic</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>VCV003132975</t>
+          <t>VCV001173081</t>
         </is>
       </c>
       <c r="H4" t="n">
@@ -621,11 +621,19 @@
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>SCV004911795: LP, Ambry Genetics, 2023-11-20 [The c.507C&gt;G (p.H169Q) alteration is located in exon 7 (coding exon 7) of the BAP1 gene. This alteration results from a C to G substitution at nucleotide position 507, causing the histidine (H) at amino acid position 169 to be replaced by a glutamine (Q). _x000D_ _x000D_ for BAP1-related neurodevelopmental disorder; however, its clinical significance for BAP1-related tumor predisposition syndrome is uncertain. This variant was not reported in population-based cohorts in the Genome Aggregation Database (gnomAD). Another alteration at the same codon, c.506A&gt;G (p.H169R), has been detected as de novo in two individuals with a syndromic form of intellectual disability and/or developmental delay (K&amp;uuml;ry, 2022). This amino acid position is highly conserved in available vertebrate species. This missense alteration is located in a region that has a low rate of benign missense variation (Lek, 2016; Firth, 2009). Based on internal structural analysis, the variant disrupts a catalytic site (K&amp;u]</t>
-        </is>
-      </c>
-      <c r="J4" t="inlineStr"/>
-      <c r="K4" t="inlineStr"/>
+          <t>SCV001738372: P, Cond: Neurodevelopmental disorder, MedGenet, 2021-06-22 [de novo; affected: yes]</t>
+        </is>
+      </c>
+      <c r="J4" t="inlineStr">
+        <is>
+          <t>F5 (Sex: female; Age_at_last_investigation: 11 years 5 months; Growth_failure: +; Developmental_delay_or_ID: +; severe; Seizures: +; Urogenital_kidney_anomalies: +; Feet: +; Facial_dysmorphism: +; Other_recurrent_signs: hypertrichosis)</t>
+        </is>
+      </c>
+      <c r="K4" t="inlineStr">
+        <is>
+          <t>44493 (GDX)</t>
+        </is>
+      </c>
       <c r="L4" t="inlineStr"/>
     </row>
     <row r="5">
@@ -636,33 +644,43 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>p.Ser10Arg</t>
+          <t>p.His169Gln</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>c.28A&gt;C</t>
+          <t>c.507C&gt;G</t>
         </is>
       </c>
       <c r="D5" t="n">
-        <v>-0.162408606</v>
+        <v>-0.1688213</v>
       </c>
       <c r="E5" t="inlineStr">
         <is>
           <t>Abnormal</t>
         </is>
       </c>
-      <c r="F5" t="inlineStr"/>
-      <c r="G5" t="inlineStr"/>
-      <c r="H5" t="inlineStr"/>
-      <c r="I5" t="inlineStr"/>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>Likely pathogenic</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>VCV003132975</t>
+        </is>
+      </c>
+      <c r="H5" t="n">
+        <v>1</v>
+      </c>
+      <c r="I5" t="inlineStr">
+        <is>
+          <t>SCV004911795: LP, Ambry Genetics, 2023-11-20 [The c.507C&gt;G (p.H169Q) alteration is located in exon 7 (coding exon 7) of the BAP1 gene. This alteration results from a C to G substitution at nucleotide position 507, causing the histidine (H) at amino acid position 169 to be replaced by a glutamine (Q). _x000D_ _x000D_ for BAP1-related neurodevelopmental disorder; however, its clinical significance for BAP1-related tumor predisposition syndrome is uncertain. This variant was not reported in population-based cohorts in the Genome Aggregation Database (gnomAD). Another alteration at the same codon, c.506A&gt;G (p.H169R), has been detected as de novo in two individuals with a syndromic form of intellectual disability and/or developmental delay (K&amp;uuml;ry, 2022). This amino acid position is highly conserved in available vertebrate species. This missense alteration is located in a region that has a low rate of benign missense variation (Lek, 2016; Firth, 2009). Based on internal structural analysis, the variant disrupts a catalytic site (K&amp;u]</t>
+        </is>
+      </c>
       <c r="J5" t="inlineStr"/>
       <c r="K5" t="inlineStr"/>
-      <c r="L5" t="inlineStr">
-        <is>
-          <t>Patient 534278 (Pathogenic; 46XY; De novo (parentage confirmed)) [Bifid uvula; Broad eyebrow; Disproportionate short stature; Intellectual disability; Osteoporosis]</t>
-        </is>
-      </c>
+      <c r="L5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -672,47 +690,33 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>p.Cys91Gly</t>
+          <t>p.Ser10Arg</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>c.271T&gt;G</t>
+          <t>c.28A&gt;C</t>
         </is>
       </c>
       <c r="D6" t="n">
-        <v>-0.160607177</v>
+        <v>-0.162408606</v>
       </c>
       <c r="E6" t="inlineStr">
         <is>
           <t>Abnormal</t>
         </is>
       </c>
-      <c r="F6" t="inlineStr">
-        <is>
-          <t>Uncertain significance</t>
-        </is>
-      </c>
-      <c r="G6" t="inlineStr">
-        <is>
-          <t>VCV001173082</t>
-        </is>
-      </c>
-      <c r="H6" t="n">
-        <v>1</v>
-      </c>
-      <c r="I6" t="inlineStr">
-        <is>
-          <t>SCV001738373: P, Cond: Neurodevelopmental disorder, MedGenet, 2021-06-22 [de novo; affected: yes]</t>
-        </is>
-      </c>
-      <c r="J6" t="inlineStr">
-        <is>
-          <t>F6 (Sex: female; Age_at_last_investigation: 15 years; Growth_failure: +; Developmental_delay_or_ID: +; severe; Behavioral_anomalies: +; ASD; Eye_anomalies: +; Hands: +; Feet: +; Feeding_difficulties: +; Facial_dysmorphism: +; Other_recurrent_signs: hypertrichosis)</t>
-        </is>
-      </c>
+      <c r="F6" t="inlineStr"/>
+      <c r="G6" t="inlineStr"/>
+      <c r="H6" t="inlineStr"/>
+      <c r="I6" t="inlineStr"/>
+      <c r="J6" t="inlineStr"/>
       <c r="K6" t="inlineStr"/>
-      <c r="L6" t="inlineStr"/>
+      <c r="L6" t="inlineStr">
+        <is>
+          <t>Patient 534278 (Pathogenic; 46XY; De novo (parentage confirmed)) [Bifid uvula; Broad eyebrow; Disproportionate short stature; Intellectual disability; Osteoporosis]</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -722,16 +726,16 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>p.Pro12Ala</t>
+          <t>p.Cys91Gly</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>c.34C&gt;G</t>
+          <t>c.271T&gt;G</t>
         </is>
       </c>
       <c r="D7" t="n">
-        <v>-0.152002451</v>
+        <v>-0.160607177</v>
       </c>
       <c r="E7" t="inlineStr">
         <is>
@@ -740,12 +744,12 @@
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>Likely pathogenic</t>
+          <t>Uncertain significance</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>VCV001173077</t>
+          <t>VCV001173082</t>
         </is>
       </c>
       <c r="H7" t="n">
@@ -753,12 +757,12 @@
       </c>
       <c r="I7" t="inlineStr">
         <is>
-          <t>SCV001738368: P, Cond: Neurodevelopmental disorder, MedGenet, 2021-06-22 [de novo; affected: yes]; SCV002098942: P, Cond: KURY-ISIDOR SYNDROME, OMIM, 2022-02-24</t>
+          <t>SCV001738373: P, Cond: Neurodevelopmental disorder, MedGenet, 2021-06-22 [de novo; affected: yes]</t>
         </is>
       </c>
       <c r="J7" t="inlineStr">
         <is>
-          <t>F2 (Sex: male; Age_at_last_investigation: 3 years; Developmental_delay_or_ID: +; Behavioral_anomalies: +; ASD; Cardiac_anomalies: +; Eye_anomalies: +; Hands: +; Facial_dysmorphism: +; Other_recurrent_signs: hearing loss)</t>
+          <t>F6 (Sex: female; Age_at_last_investigation: 15 years; Growth_failure: +; Developmental_delay_or_ID: +; severe; Behavioral_anomalies: +; ASD; Eye_anomalies: +; Hands: +; Feet: +; Feeding_difficulties: +; Facial_dysmorphism: +; Other_recurrent_signs: hypertrichosis)</t>
         </is>
       </c>
       <c r="K7" t="inlineStr"/>
@@ -831,7 +835,7 @@
         </is>
       </c>
       <c r="D9" t="n">
-        <v>-0.135425214</v>
+        <v>-0.137253385</v>
       </c>
       <c r="E9" t="inlineStr">
         <is>
@@ -972,35 +976,45 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>p.Tyr33Ser</t>
+          <t>p.Arg59Pro</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>c.98A&gt;C</t>
+          <t>c.176G&gt;C</t>
         </is>
       </c>
       <c r="D12" t="n">
-        <v>-0.071735567</v>
+        <v>-0.102311315</v>
       </c>
       <c r="E12" t="inlineStr">
         <is>
           <t>Abnormal</t>
         </is>
       </c>
-      <c r="F12" t="inlineStr"/>
-      <c r="G12" t="inlineStr"/>
-      <c r="H12" t="inlineStr"/>
-      <c r="I12" t="inlineStr"/>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>Pathogenic</t>
+        </is>
+      </c>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>VCV001173080</t>
+        </is>
+      </c>
+      <c r="H12" t="n">
+        <v>1</v>
+      </c>
+      <c r="I12" t="inlineStr">
+        <is>
+          <t>SCV001738371: P, Cond: Neurodevelopmental disorder, MedGenet, 2021-06-22 [de novo; affected: yes]</t>
+        </is>
+      </c>
       <c r="J12" t="inlineStr"/>
-      <c r="K12" t="inlineStr">
-        <is>
-          <t>DDD13k.07819 (DDD)</t>
-        </is>
-      </c>
+      <c r="K12" t="inlineStr"/>
       <c r="L12" t="inlineStr">
         <is>
-          <t>Patient 272983 (Likely pathogenic; 46XX; De novo (parentage confirmed); ACMG: PM2;PP3;PS2) [Aggressive behavior; Cafe-au-lait spot; Downturned corners of mouth; High palate; Long philtrum; Low posterior hairline; Short neck; Specific learning disability; Triphalangeal thumb]</t>
+          <t>Patient 550703 (Likely pathogenic; 46XX; De novo (parentage confirmed))</t>
         </is>
       </c>
     </row>
@@ -1012,16 +1026,16 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>p.Ala92Val</t>
+          <t>p.Pro12Ala</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>c.275C&gt;T</t>
+          <t>c.34C&gt;G</t>
         </is>
       </c>
       <c r="D13" t="n">
-        <v>-0.061896707</v>
+        <v>-0.07773922</v>
       </c>
       <c r="E13" t="inlineStr">
         <is>
@@ -1030,23 +1044,27 @@
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>Pathogenic/Likely pathogenic</t>
+          <t>Likely pathogenic</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>VCV002681785</t>
+          <t>VCV001173077</t>
         </is>
       </c>
       <c r="H13" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="I13" t="inlineStr">
         <is>
-          <t>SCV005420942: LP, IMGAG, 2024-12-09 [affected: yes; clinical features: Strabismus, Irritability, Delayed speech and language development, Global developmental delay, Motor delay, Disproportionate short stature, Pain insensitivity, Thinning of lateral eyebrow, Recurrent hand flapping, Self-injurious behavior]</t>
-        </is>
-      </c>
-      <c r="J13" t="inlineStr"/>
+          <t>SCV001738368: P, Cond: Neurodevelopmental disorder, MedGenet, 2021-06-22 [de novo; affected: yes]; SCV002098942: P, Cond: KURY-ISIDOR SYNDROME, OMIM, 2022-02-24</t>
+        </is>
+      </c>
+      <c r="J13" t="inlineStr">
+        <is>
+          <t>F2 (Sex: male; Age_at_last_investigation: 3 years; Developmental_delay_or_ID: +; Behavioral_anomalies: +; ASD; Cardiac_anomalies: +; Eye_anomalies: +; Hands: +; Facial_dysmorphism: +; Other_recurrent_signs: hearing loss)</t>
+        </is>
+      </c>
       <c r="K13" t="inlineStr"/>
       <c r="L13" t="inlineStr"/>
     </row>
@@ -1058,43 +1076,37 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>p.Ser10Gly</t>
+          <t>p.Tyr33Ser</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>c.28A&gt;G</t>
+          <t>c.98A&gt;C</t>
         </is>
       </c>
       <c r="D14" t="n">
-        <v>-0.056445873</v>
+        <v>-0.071735567</v>
       </c>
       <c r="E14" t="inlineStr">
         <is>
           <t>Abnormal</t>
         </is>
       </c>
-      <c r="F14" t="inlineStr">
-        <is>
-          <t>Likely pathogenic</t>
-        </is>
-      </c>
-      <c r="G14" t="inlineStr">
-        <is>
-          <t>VCV003377067</t>
-        </is>
-      </c>
-      <c r="H14" t="n">
-        <v>1</v>
-      </c>
-      <c r="I14" t="inlineStr">
-        <is>
-          <t>SCV005399747: LP, VCGS, 2024-10-09 [affected: yes; Based on the classification scheme VCGS_Germline_v1.3.4, this variant is classified as Likely pathogenic. Following criteria are met: 0102 - Loss of function is a known mechanism of disease in this gene and is associated with tumour predisposition syndrome 1 (MIM#614327). Loss of function has also been reported for missense variants associated with Kury-Isidor syndrome (MIM#619762), however dominant negative has not been excluded (PMID: 35051358). (I) 0107 - This gene is associated with autosomal dominant disease. Only missense variants have been reported for Kury-Isidor, while all variant types have been reported for tumour predisposition syndrome (PMID: 38506155). (I) 0115 - Variants in this gene are known to have variable expressivity. Kury-Isidor syndrome is known to be widely variable (OMIM). (I) 0200 - Variant is predicted to result in a missense amino acid change from serine to glycine. (I) 0251 - This variant is heterozygous. (I) 0301 - Variant is absent from gnomAD (both v2 an]</t>
-        </is>
-      </c>
+      <c r="F14" t="inlineStr"/>
+      <c r="G14" t="inlineStr"/>
+      <c r="H14" t="inlineStr"/>
+      <c r="I14" t="inlineStr"/>
       <c r="J14" t="inlineStr"/>
-      <c r="K14" t="inlineStr"/>
-      <c r="L14" t="inlineStr"/>
+      <c r="K14" t="inlineStr">
+        <is>
+          <t>DDD13k.07819 (DDD)</t>
+        </is>
+      </c>
+      <c r="L14" t="inlineStr">
+        <is>
+          <t>Patient 272983 (Likely pathogenic; 46XX; De novo (parentage confirmed); ACMG: PM2;PP3;PS2) [Aggressive behavior; Cafe-au-lait spot; Downturned corners of mouth; High palate; Long philtrum; Low posterior hairline; Short neck; Specific learning disability; Triphalangeal thumb]</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -1104,38 +1116,38 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>p.Arg60Gln</t>
+          <t>p.Ala92Val</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>c.179G&gt;A</t>
+          <t>c.275C&gt;T</t>
         </is>
       </c>
       <c r="D15" t="n">
-        <v>-0.018285555</v>
+        <v>-0.061896707</v>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>Normal</t>
+          <t>Abnormal</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>Conflicting classifications of pathogenicity</t>
+          <t>Pathogenic/Likely pathogenic</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>VCV000489626</t>
+          <t>VCV002681785</t>
         </is>
       </c>
       <c r="H15" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="I15" t="inlineStr">
         <is>
-          <t>SCV006277912: LP, IMGAG, 2025-07-10 [affected: yes; clinical features: Low frustration tolerance, Delayed speech and language development, Hypertrichosis, Global developmental delay, Motor delay, Small for gestational age, Short stature, Attention deficit hyperactivity disorder, Feeding difficulties in infancy, Neurodevelopmental delay, Difficulty walking on uneven ground, Hand flapping]</t>
+          <t>SCV005420942: LP, IMGAG, 2024-12-09 [affected: yes; clinical features: Strabismus, Irritability, Delayed speech and language development, Global developmental delay, Motor delay, Disproportionate short stature, Pain insensitivity, Thinning of lateral eyebrow, Recurrent hand flapping, Self-injurious behavior]</t>
         </is>
       </c>
       <c r="J15" t="inlineStr"/>
@@ -1150,16 +1162,16 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>p.Arg59Pro</t>
+          <t>p.Ser10Gly</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>c.176G&gt;C</t>
+          <t>c.28A&gt;G</t>
         </is>
       </c>
       <c r="D16" t="n">
-        <v>0.000595509</v>
+        <v>-0.056445873</v>
       </c>
       <c r="E16" t="inlineStr">
         <is>
@@ -1168,12 +1180,12 @@
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>Pathogenic</t>
+          <t>Likely pathogenic</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>VCV001173080</t>
+          <t>VCV003377067</t>
         </is>
       </c>
       <c r="H16" t="n">
@@ -1181,16 +1193,12 @@
       </c>
       <c r="I16" t="inlineStr">
         <is>
-          <t>SCV001738371: P, Cond: Neurodevelopmental disorder, MedGenet, 2021-06-22 [de novo; affected: yes]</t>
+          <t>SCV005399747: LP, VCGS, 2024-10-09 [affected: yes; Based on the classification scheme VCGS_Germline_v1.3.4, this variant is classified as Likely pathogenic. Following criteria are met: 0102 - Loss of function is a known mechanism of disease in this gene and is associated with tumour predisposition syndrome 1 (MIM#614327). Loss of function has also been reported for missense variants associated with Kury-Isidor syndrome (MIM#619762), however dominant negative has not been excluded (PMID: 35051358). (I) 0107 - This gene is associated with autosomal dominant disease. Only missense variants have been reported for Kury-Isidor, while all variant types have been reported for tumour predisposition syndrome (PMID: 38506155). (I) 0115 - Variants in this gene are known to have variable expressivity. Kury-Isidor syndrome is known to be widely variable (OMIM). (I) 0200 - Variant is predicted to result in a missense amino acid change from serine to glycine. (I) 0251 - This variant is heterozygous. (I) 0301 - Variant is absent from gnomAD (both v2 an]</t>
         </is>
       </c>
       <c r="J16" t="inlineStr"/>
       <c r="K16" t="inlineStr"/>
-      <c r="L16" t="inlineStr">
-        <is>
-          <t>Patient 550703 (Likely pathogenic; 46XX; De novo (parentage confirmed))</t>
-        </is>
-      </c>
+      <c r="L16" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -1200,51 +1208,43 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>p.Asn229Lys</t>
+          <t>p.Arg60Gln</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>c.687C&gt;A</t>
+          <t>c.179G&gt;A</t>
         </is>
       </c>
       <c r="D17" t="n">
-        <v>0.00165034</v>
+        <v>-0.018285555</v>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>Abnormal</t>
+          <t>Normal</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>Likely pathogenic</t>
+          <t>Conflicting classifications of pathogenicity</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>VCV002429331</t>
+          <t>VCV000489626</t>
         </is>
       </c>
       <c r="H17" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="I17" t="inlineStr">
         <is>
-          <t>SCV003799185: LP, IHG-UKRWTH, 2023-02-09 [de novo; affected: yes; To our knowledge, the variant has not yet been described in the literature. Küry S. et al. (2022) describe 11 individuals with a similar phenotype to our patient with de novo missense variants in BAP1, which are also located d in a protein domain that encodes for a ubiquitin carboxyl-terminal hydrolase (peptidase C12) and the papain-like cysteine ​​peptidase superfamily. Functional studies of these variants show that they alter chromatin remodeling through abnormal histone ubiquitination and result in transcriptional dysregulation of developmental genes. (PMID: 35051358) These findings suggest that this could also lead to defective histone ubiquitination in the variant described here.]; SCV006550944: LP, UDN, 2025-06-11 [de novo; affected: yes; clinical features: Hearing impairment, Short neck, Cataract, Retinal detachment, Leukocoria, Microphthalmia, Shallow anterior chamber, Brachydactyly, Global developmental delay, Sandal gap, Bilateral retinal detachment, Hallux valgus]</t>
+          <t>SCV006277912: LP, IMGAG, 2025-07-10 [affected: yes; clinical features: Low frustration tolerance, Delayed speech and language development, Hypertrichosis, Global developmental delay, Motor delay, Small for gestational age, Short stature, Attention deficit hyperactivity disorder, Feeding difficulties in infancy, Neurodevelopmental delay, Difficulty walking on uneven ground, Hand flapping]</t>
         </is>
       </c>
       <c r="J17" t="inlineStr"/>
-      <c r="K17" t="inlineStr">
-        <is>
-          <t>DDD13k.05634 (DDD)</t>
-        </is>
-      </c>
-      <c r="L17" t="inlineStr">
-        <is>
-          <t>Patient 264575 (46XY; De novo (parentage confirmed)) [3-4 finger osseus syndactyly; Abnormal forehead morphology; Abnormal nail morphology; Broad forehead; Cutaneous finger syndactyly; Delayed gross motor development; Delayed speech and language development; Global developmental delay; Hypermetropia; Microdontia; Short stature; Upslanted palpebral fissure]</t>
-        </is>
-      </c>
+      <c r="K17" t="inlineStr"/>
+      <c r="L17" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -1263,7 +1263,7 @@
         </is>
       </c>
       <c r="D18" t="n">
-        <v>0.004099673</v>
+        <v>0.00336388</v>
       </c>
       <c r="E18" t="inlineStr">
         <is>
@@ -1313,7 +1313,7 @@
         </is>
       </c>
       <c r="D19" t="n">
-        <v>0.010065746</v>
+        <v>0.007149731</v>
       </c>
       <c r="E19" t="inlineStr">
         <is>

</xml_diff>